<commit_message>
housekeep-db: The appearance of excel format improved
</commit_message>
<xml_diff>
--- a/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-ja_sample.xlsx
+++ b/ecuacion-tool-housekeep-db/excel-format/housekeep-db_fmt-v2.0.0-ja_sample.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tools/ecuacion-tool-housekeep-db/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B60B1A6A-CF2D-C943-80EE-B2260C21A959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7C33A7-38BC-3248-9A0D-AD6F9AACB77F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16600" activeTab="1" xr2:uid="{8AED4C0F-E98F-E547-A0B0-59373B747A30}"/>
+    <workbookView xWindow="2500" yWindow="500" windowWidth="28800" windowHeight="16600" xr2:uid="{8AED4C0F-E98F-E547-A0B0-59373B747A30}"/>
   </bookViews>
   <sheets>
     <sheet name="fmt変更履歴" sheetId="8" r:id="rId1"/>
-    <sheet name="Info" sheetId="5" r:id="rId2"/>
+    <sheet name="Info" sheetId="5" state="hidden" r:id="rId2"/>
     <sheet name="dropdown" sheetId="15" state="hidden" r:id="rId3"/>
     <sheet name="DB接続設定" sheetId="4" r:id="rId4"/>
     <sheet name="housekeep DB設定" sheetId="10" r:id="rId5"/>
@@ -54,7 +54,7 @@
     <author>tc={7D829323-4655-CD44-9CAF-FB0BE1358339}</author>
   </authors>
   <commentList>
-    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{7D829323-4655-CD44-9CAF-FB0BE1358339}">
+    <comment ref="F4" authorId="0" shapeId="0" xr:uid="{7D829323-4655-CD44-9CAF-FB0BE1358339}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="79">
   <si>
     <t>value</t>
     <phoneticPr fontId="1"/>
@@ -408,36 +408,6 @@
   </si>
   <si>
     <t>田中</t>
-  </si>
-  <si>
-    <t>※「論理廃止：更新用ユーザIDカラム名」、「論理廃止：更新用ユーザIDカラム型リテラル記号」、「論理廃止：更新用ユーザIDカラム値」は、「論理廃止／削除」が「削除」の場合は空欄、「論理廃止」の場合は任意。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>※「接続url : schema」は、default schema（ユーザ名と同じスキーマ）でない場合のみ設定</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>※「論理廃止：更新用timestampカラム名」は、「論理廃止／削除」が「削除」の場合は空欄、「論理廃止」の場合は任意。論理廃止時にtimestampを更新する項目がある場合に指定。値は自動で現在時刻を設定。</t>
-    <rPh sb="26" eb="27">
-      <t xml:space="preserve">サクジョ </t>
-    </rPh>
-    <rPh sb="32" eb="34">
-      <t xml:space="preserve">クウラン </t>
-    </rPh>
-    <rPh sb="45" eb="47">
-      <t xml:space="preserve">ニンイ。 </t>
-    </rPh>
-    <rPh sb="57" eb="58">
-      <t xml:space="preserve">アタイハジドウデ </t>
-    </rPh>
-    <rPh sb="62" eb="66">
-      <t xml:space="preserve">ゲンザイジコクヲシテイ </t>
-    </rPh>
-    <rPh sb="67" eb="69">
-      <t xml:space="preserve">セッテイ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>v.1.2.0</t>
@@ -485,9 +455,6 @@
       ・論理廃止：カラム名 -&gt; 削除フラグカラム名</t>
   </si>
   <si>
-    <t>※「期間経過チェック用：timestampカラム名」、「期間経過チェック用：timestampカラム型」、「期間経過チェック用：timestamp要経過日数」は任意。ただし、全て空欄か全て入力のいずれか。</t>
-  </si>
-  <si>
     <t>論理廃止：更新用ユーザIDカラム名</t>
   </si>
   <si>
@@ -507,36 +474,6 @@
   </si>
   <si>
     <t>ja</t>
-  </si>
-  <si>
-    <t>必須</t>
-  </si>
-  <si>
-    <t>任意</t>
-  </si>
-  <si>
-    <t>「削除」の場合は任意、「論理廃止」の場合は必須</t>
-  </si>
-  <si>
-    <t>「削除」の場合は空欄、「論理廃止」の場合は任意</t>
-  </si>
-  <si>
-    <t>　指定せずに論理廃止／削除する場合、レコード作成・更新からの期間経過を加味せず削除。</t>
-  </si>
-  <si>
-    <t>※「削除フラグカラム名」は、「削除」の場合で本項目を指定すると、指定のカラムが"true"の場合のみ削除実施される</t>
-  </si>
-  <si>
-    <t>　（削除フラグカラムはbool型のみ対応可）</t>
-  </si>
-  <si>
-    <t>※「論理廃止：更新用timestampカラム名」は、論理廃止時にtimestampを更新する項目がある場合に指定。値は自動で現在時刻を設定。</t>
-  </si>
-  <si>
-    <t>※「論理廃止：更新用ユーザIDカラム名」、「論理廃止：更新用ユーザIDカラム型リテラル記号」、「論理廃止：更新用ユーザIDカラム値」は、論理廃止時にユーザID項目を更新する項目がある場合に指定。</t>
-  </si>
-  <si>
-    <t>　全て空欄か全て入力のいずれか。</t>
   </si>
   <si>
     <t>処理ID</t>
@@ -576,19 +513,10 @@
     <t>データ検索条件設定</t>
   </si>
   <si>
-    <t>※「削除フラグカラム名」は、「housekeep DB設定」シートの「論理廃止／削除」が「論理廃止」の場合は必須、「削除」の場合は任意。「削除」の場合で本項目を指定すると、指定のカラムが"true"の場合のみ削除実施される</t>
-  </si>
-  <si>
-    <t>　全て空欄か、全て空欄でない状態である必要あり。</t>
-  </si>
-  <si>
     <t>論理廃止 / 削除</t>
   </si>
   <si>
     <t>論理廃止 / 削除（内部値）</t>
-  </si>
-  <si>
-    <t>変更禁止！</t>
   </si>
   <si>
     <t>関連テーブル処理パターン（内部値）</t>
@@ -604,10 +532,13 @@
 　- 1行目のコメントを削除</t>
   </si>
   <si>
-    <t>論理廃止／削除</t>
-  </si>
-  <si>
     <t>2.0.0</t>
+  </si>
+  <si>
+    <t>期間経過チェック項目</t>
+  </si>
+  <si>
+    <t>論理廃止用項目</t>
   </si>
 </sst>
 </file>
@@ -704,7 +635,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -728,26 +659,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFAB7942"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD883FF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.34998626667073579"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -770,6 +683,78 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="hair">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color theme="0"/>
+      </left>
+      <right style="hair">
+        <color theme="0"/>
+      </right>
+      <top style="hair">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color theme="0"/>
+      </left>
+      <right style="hair">
+        <color theme="0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color theme="0"/>
+      </left>
+      <right style="hair">
+        <color theme="0"/>
+      </right>
+      <top style="hair">
+        <color theme="0"/>
+      </top>
+      <bottom style="hair">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color theme="0"/>
+      </top>
+      <bottom style="hair">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -783,7 +768,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -849,37 +834,46 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1084,6 +1078,22 @@
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color theme="0"/>
+        </left>
+        <right style="hair">
+          <color theme="0"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="hair">
+          <color theme="0"/>
+        </vertical>
+        <horizontal style="hair">
+          <color theme="0"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1154,6 +1164,310 @@
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color theme="0"/>
+        </left>
+        <right style="hair">
+          <color theme="0"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="hair">
+          <color theme="0"/>
+        </vertical>
+        <horizontal style="hair">
+          <color theme="0"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color theme="0"/>
+        </left>
+        <right style="hair">
+          <color theme="0"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="hair">
+          <color theme="0"/>
+        </vertical>
+        <horizontal style="hair">
+          <color theme="0"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1407,278 +1721,6 @@
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1830,76 +1872,76 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{22FC8765-21CB-4449-8794-6F7BB0DF5CF4}" name="テーブル5" displayName="テーブル5" ref="A3:D9" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{22FC8765-21CB-4449-8794-6F7BB0DF5CF4}" name="テーブル5" displayName="テーブル5" ref="A3:D9" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A3:D9" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E4142994-3892-C340-9A65-88F80365D8CE}" name="日付" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{35BACA5E-E809-0844-BAB8-78CB7B6B343E}" name="バージョン" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{C4E826C9-5641-E048-9706-B0754516BA47}" name="修正事項" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{10D446C7-4721-E74C-863B-894EBEBABA4B}" name="修正者" dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{E4142994-3892-C340-9A65-88F80365D8CE}" name="日付" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{35BACA5E-E809-0844-BAB8-78CB7B6B343E}" name="バージョン" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{C4E826C9-5641-E048-9706-B0754516BA47}" name="修正事項" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{10D446C7-4721-E74C-863B-894EBEBABA4B}" name="修正者" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{24155060-B8ED-8845-8CC4-DA9C5F0847AB}" name="テーブル4" displayName="テーブル4" ref="A1:B3" totalsRowShown="0" headerRowDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{24155060-B8ED-8845-8CC4-DA9C5F0847AB}" name="テーブル4" displayName="テーブル4" ref="A1:B3" totalsRowShown="0" headerRowDxfId="32">
   <autoFilter ref="A1:B3" xr:uid="{24155060-B8ED-8845-8CC4-DA9C5F0847AB}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{98E4E7E5-8F2D-A64D-A202-DFFC12164331}" name="item" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{E3BF9435-59E2-8948-93E9-5462EEBA2F6D}" name="value" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{98E4E7E5-8F2D-A64D-A202-DFFC12164331}" name="item" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{E3BF9435-59E2-8948-93E9-5462EEBA2F6D}" name="value" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DD7B5D78-5E9B-DE4B-B691-1DF452AB1374}" name="テーブル3" displayName="テーブル3" ref="A5:I6" insertRow="1" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
-  <autoFilter ref="A5:I6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DD7B5D78-5E9B-DE4B-B691-1DF452AB1374}" name="テーブル3" displayName="テーブル3" ref="A4:I5" insertRow="1" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+  <autoFilter ref="A4:I5" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{6F9607F2-5B3B-AC43-9B81-3332FF1A0DAD}" name="DB接続ID" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{EB1F7206-30E2-EA43-A8CF-9AD4F9A14E33}" name="driver名" dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{4D55D82B-BDD3-2B46-A21D-0450B9F1910B}" name="接続url : protocol" dataDxfId="42" dataCellStyle="標準 2"/>
-    <tableColumn id="4" xr3:uid="{84D0845B-C5EE-9047-A1AB-EE336A75EBAD}" name="接続url : サーバ" dataDxfId="41" dataCellStyle="標準 2"/>
-    <tableColumn id="5" xr3:uid="{6197D9F5-186B-D44E-ADCB-89378D8B3702}" name="接続url : port" dataDxfId="40" dataCellStyle="標準 2"/>
-    <tableColumn id="6" xr3:uid="{26B865D4-D13A-9C4C-B104-C634122F988F}" name="接続url : database" dataDxfId="39" dataCellStyle="標準 2"/>
-    <tableColumn id="7" xr3:uid="{046864C3-26A2-7B44-B07A-EAB68FAF2EEA}" name="接続url : schema" dataDxfId="38" dataCellStyle="標準 2"/>
-    <tableColumn id="8" xr3:uid="{4A5FE8C4-A0F3-3E4A-9BB5-642C226504CF}" name="ユーザ名" dataDxfId="37" dataCellStyle="標準 2"/>
-    <tableColumn id="9" xr3:uid="{6A963E93-AA2B-944F-A127-0CD6F7E61369}" name="password" dataDxfId="36" dataCellStyle="標準 2"/>
+    <tableColumn id="1" xr3:uid="{6F9607F2-5B3B-AC43-9B81-3332FF1A0DAD}" name="DB接続ID" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{EB1F7206-30E2-EA43-A8CF-9AD4F9A14E33}" name="driver名" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{4D55D82B-BDD3-2B46-A21D-0450B9F1910B}" name="接続url : protocol" dataDxfId="25" dataCellStyle="標準 2"/>
+    <tableColumn id="4" xr3:uid="{84D0845B-C5EE-9047-A1AB-EE336A75EBAD}" name="接続url : サーバ" dataDxfId="24" dataCellStyle="標準 2"/>
+    <tableColumn id="5" xr3:uid="{6197D9F5-186B-D44E-ADCB-89378D8B3702}" name="接続url : port" dataDxfId="23" dataCellStyle="標準 2"/>
+    <tableColumn id="6" xr3:uid="{26B865D4-D13A-9C4C-B104-C634122F988F}" name="接続url : database" dataDxfId="22" dataCellStyle="標準 2"/>
+    <tableColumn id="7" xr3:uid="{046864C3-26A2-7B44-B07A-EAB68FAF2EEA}" name="接続url : schema" dataDxfId="21" dataCellStyle="標準 2"/>
+    <tableColumn id="8" xr3:uid="{4A5FE8C4-A0F3-3E4A-9BB5-642C226504CF}" name="ユーザ名" dataDxfId="20" dataCellStyle="標準 2"/>
+    <tableColumn id="9" xr3:uid="{6A963E93-AA2B-944F-A127-0CD6F7E61369}" name="password" dataDxfId="19" dataCellStyle="標準 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61C29F33-44CC-B14C-8562-09C29609B4D7}" name="テーブル32" displayName="テーブル32" ref="A5:O6" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
-  <autoFilter ref="A5:O6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61C29F33-44CC-B14C-8562-09C29609B4D7}" name="テーブル32" displayName="テーブル32" ref="A4:O5" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+  <autoFilter ref="A4:O5" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{CBD51E9F-618C-754C-8BA6-0B46FCE3F82F}" name="処理ID" dataDxfId="33"/>
-    <tableColumn id="12" xr3:uid="{5E33A481-4C3C-A049-B253-3EC944DDB6EC}" name="DB接続ID" dataDxfId="32" dataCellStyle="標準 2"/>
-    <tableColumn id="2" xr3:uid="{AADC801E-ABC4-9E4F-8EFF-3383030B2A4B}" name="論理廃止 / 削除" dataDxfId="31"/>
-    <tableColumn id="15" xr3:uid="{F58118F0-6716-6C42-853A-3FBAEE07F4E8}" name="論理廃止 / 削除（内部値）" dataDxfId="30">
+    <tableColumn id="1" xr3:uid="{CBD51E9F-618C-754C-8BA6-0B46FCE3F82F}" name="処理ID" dataDxfId="53"/>
+    <tableColumn id="12" xr3:uid="{5E33A481-4C3C-A049-B253-3EC944DDB6EC}" name="DB接続ID" dataDxfId="52" dataCellStyle="標準 2"/>
+    <tableColumn id="2" xr3:uid="{AADC801E-ABC4-9E4F-8EFF-3383030B2A4B}" name="論理廃止 / 削除" dataDxfId="51"/>
+    <tableColumn id="15" xr3:uid="{F58118F0-6716-6C42-853A-3FBAEE07F4E8}" name="論理廃止 / 削除（内部値）" dataDxfId="50">
       <calculatedColumnFormula array="1">_xlfn.IFS(テーブル32[[#This Row],[論理廃止 / 削除]]="論理廃止","SOFT_DELETE",テーブル32[[#This Row],[論理廃止 / 削除]]="削除","HARD_DELETE",TRUE,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{6C98AD64-A3D3-F44E-A881-8EFCEA1F9F67}" name="テーブル名" dataDxfId="29" dataCellStyle="標準 2"/>
-    <tableColumn id="4" xr3:uid="{A38A3149-447A-8548-9729-49CE9E074B36}" name="IDカラム名" dataDxfId="28" dataCellStyle="標準 2"/>
-    <tableColumn id="10" xr3:uid="{B15AF0F8-272C-B943-9D75-81A8797BC598}" name="IDカラム型リテラル記号" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{6FE6A1FF-15C9-7545-B254-7B2C29EF168D}" name="期間経過チェック用：timestampカラム名" dataDxfId="26" dataCellStyle="標準 2"/>
-    <tableColumn id="11" xr3:uid="{BF075527-A2E7-834B-AD05-1A2D9E3BA0AD}" name="期間経過チェック用：timestampカラム型" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{94EB7746-8D75-EE47-A2F3-81D397D26AE1}" name="期間経過チェック用：timestamp要経過日数" dataDxfId="24" dataCellStyle="標準 2"/>
-    <tableColumn id="7" xr3:uid="{62ADB4F3-1C59-7F4B-819E-B49B0ABB889C}" name="削除フラグカラム名" dataDxfId="23" dataCellStyle="標準 2"/>
-    <tableColumn id="8" xr3:uid="{0EB6A694-7E00-B64C-AF69-22B6C7E1C560}" name="論理廃止：更新用timestampカラム名" dataDxfId="22" dataCellStyle="標準 2"/>
-    <tableColumn id="9" xr3:uid="{0A6924E1-C0CB-AF40-A208-E0E96A257245}" name="論理廃止：更新用ユーザIDカラム名" dataDxfId="21" dataCellStyle="標準 2"/>
-    <tableColumn id="14" xr3:uid="{93BF3B4F-D2E8-A640-A768-A230439878D9}" name="論理廃止：更新用ユーザIDカラム型リテラル記号" dataDxfId="20" dataCellStyle="標準 2"/>
-    <tableColumn id="13" xr3:uid="{DE6ACC44-9137-0840-9711-E0D04FCC851F}" name="論理廃止：更新用ユーザIDカラム値" dataDxfId="19" dataCellStyle="標準 2"/>
+    <tableColumn id="3" xr3:uid="{6C98AD64-A3D3-F44E-A881-8EFCEA1F9F67}" name="テーブル名" dataDxfId="49" dataCellStyle="標準 2"/>
+    <tableColumn id="4" xr3:uid="{A38A3149-447A-8548-9729-49CE9E074B36}" name="IDカラム名" dataDxfId="48" dataCellStyle="標準 2"/>
+    <tableColumn id="10" xr3:uid="{B15AF0F8-272C-B943-9D75-81A8797BC598}" name="IDカラム型リテラル記号" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{6FE6A1FF-15C9-7545-B254-7B2C29EF168D}" name="期間経過チェック用：timestampカラム名" dataDxfId="46" dataCellStyle="標準 2"/>
+    <tableColumn id="11" xr3:uid="{BF075527-A2E7-834B-AD05-1A2D9E3BA0AD}" name="期間経過チェック用：timestampカラム型" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{94EB7746-8D75-EE47-A2F3-81D397D26AE1}" name="期間経過チェック用：timestamp要経過日数" dataDxfId="44" dataCellStyle="標準 2"/>
+    <tableColumn id="7" xr3:uid="{62ADB4F3-1C59-7F4B-819E-B49B0ABB889C}" name="削除フラグカラム名" dataDxfId="43" dataCellStyle="標準 2"/>
+    <tableColumn id="8" xr3:uid="{0EB6A694-7E00-B64C-AF69-22B6C7E1C560}" name="論理廃止：更新用timestampカラム名" dataDxfId="42" dataCellStyle="標準 2"/>
+    <tableColumn id="9" xr3:uid="{0A6924E1-C0CB-AF40-A208-E0E96A257245}" name="論理廃止：更新用ユーザIDカラム名" dataDxfId="41" dataCellStyle="標準 2"/>
+    <tableColumn id="14" xr3:uid="{93BF3B4F-D2E8-A640-A768-A230439878D9}" name="論理廃止：更新用ユーザIDカラム型リテラル記号" dataDxfId="40" dataCellStyle="標準 2"/>
+    <tableColumn id="13" xr3:uid="{DE6ACC44-9137-0840-9711-E0D04FCC851F}" name="論理廃止：更新用ユーザIDカラム値" dataDxfId="39" dataCellStyle="標準 2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DBD8E589-22D9-8541-A9D6-F03C8FC47C4E}" name="テーブル323" displayName="テーブル323" ref="A5:D6" insertRow="1" totalsRowShown="0" headerRowDxfId="18">
-  <autoFilter ref="A5:D6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DBD8E589-22D9-8541-A9D6-F03C8FC47C4E}" name="テーブル323" displayName="テーブル323" ref="A4:D5" insertRow="1" totalsRowShown="0" headerRowDxfId="18">
+  <autoFilter ref="A4:D5" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{0B02141A-0F5F-8849-982C-6C0A6A7BEE4F}" name="処理ID" dataDxfId="17" dataCellStyle="標準 2"/>
     <tableColumn id="12" xr3:uid="{69A08ECC-4076-9E48-8CE9-3FABB073CA81}" name="条件カラム名" dataDxfId="16"/>
@@ -1911,8 +1953,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5EE7E132-481E-3140-932F-4C153EC6948B}" name="テーブル3236" displayName="テーブル3236" ref="A5:L6" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="A5:L6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5EE7E132-481E-3140-932F-4C153EC6948B}" name="テーブル3236" displayName="テーブル3236" ref="A4:L5" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A4:L5" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{65C86A53-0A13-8F47-916D-E06475BCECE3}" name="処理ID" dataDxfId="11"/>
     <tableColumn id="12" xr3:uid="{987F2B9C-94EA-9F41-A4C1-6D7606B12BAC}" name="関連テーブル処理パターン" dataDxfId="10"/>
@@ -2230,7 +2272,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="F5" dT="2024-08-31T07:19:37.97" personId="{78017D61-44A1-0A4F-9335-7121C27F2A1F}" id="{7D829323-4655-CD44-9CAF-FB0BE1358339}">
+  <threadedComment ref="F4" dT="2024-08-31T07:19:37.97" personId="{78017D61-44A1-0A4F-9335-7121C27F2A1F}" id="{7D829323-4655-CD44-9CAF-FB0BE1358339}">
     <text>実際のレコード削除時はIDカラムの値を指定して削除するために必要</text>
   </threadedComment>
 </ThreadedComments>
@@ -2303,7 +2345,7 @@
         <v>46</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>47</v>
@@ -2314,10 +2356,10 @@
         <v>45766</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>47</v>
@@ -2328,10 +2370,10 @@
         <v>45780</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>47</v>
@@ -2342,10 +2384,10 @@
         <v>46256</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>47</v>
@@ -2384,15 +2426,15 @@
         <v>2</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -2538,7 +2580,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A269F1A1-7AAA-9644-B9A4-2FF06B781584}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.83203125" style="6" bestFit="1" customWidth="1"/>
@@ -2548,7 +2590,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -2557,71 +2599,45 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="H4" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="I4" s="30"/>
+      <c r="A4" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="33" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
-        <v>49</v>
-      </c>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="H4:I4"/>
-  </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2633,7 +2649,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{789F72C4-22B4-0242-AA9D-05DCD1C7C1AF}">
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.5" style="6" customWidth="1"/>
@@ -2654,7 +2670,7 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B1" s="1"/>
     </row>
@@ -2662,150 +2678,105 @@
       <c r="A3" s="6" t="s">
         <v>26</v>
       </c>
+      <c r="H3" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3" s="34"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="35" t="s">
+        <v>78</v>
+      </c>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
+      <c r="N3" s="35"/>
+      <c r="O3" s="36"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
+      <c r="A4" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>71</v>
+      </c>
       <c r="D4" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="E4" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="I4" s="31"/>
-      <c r="J4" s="31"/>
-      <c r="K4" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="L4" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="M4" s="32"/>
-      <c r="N4" s="32"/>
-      <c r="O4" s="32"/>
+        <v>72</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" s="31" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="J4" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="K4" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="L4" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="M4" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="N4" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="O4" s="30" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="L5" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="M5" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="N5" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="O5" s="8" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8" t="str" cm="1">
-        <f t="array" ref="D6">_xlfn.IFS(テーブル32[[#This Row],[論理廃止 / 削除]]="論理廃止","SOFT_DELETE",テーブル32[[#This Row],[論理廃止 / 削除]]="削除","HARD_DELETE",TRUE,"")</f>
+      <c r="A5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8" t="str" cm="1">
+        <f t="array" ref="D5">_xlfn.IFS(テーブル32[[#This Row],[論理廃止 / 削除]]="論理廃止","SOFT_DELETE",テーブル32[[#This Row],[論理廃止 / 削除]]="削除","HARD_DELETE",TRUE,"")</f>
         <v/>
       </c>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="N6" s="8"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="6" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
-        <v>71</v>
-      </c>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="N5" s="8"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="6" t="s">
-        <v>72</v>
-      </c>
+      <c r="A12" s="19"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="19" t="s">
-        <v>73</v>
-      </c>
+      <c r="A13" s="19"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="19" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="19" t="s">
-        <v>75</v>
-      </c>
+      <c r="A14" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="L4:O4"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="E4:G4"/>
+  <mergeCells count="2">
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:O3"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6" xr:uid="{8F6F98C1-595C-9F49-B250-21CD2634841D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5" xr:uid="{8F6F98C1-595C-9F49-B250-21CD2634841D}">
       <formula1>"論理廃止,削除"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G6 N6" xr:uid="{7B8B2790-6C59-604D-89F1-3BD24DE216A5}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5 N5" xr:uid="{7B8B2790-6C59-604D-89F1-3BD24DE216A5}">
       <formula1>"quotes('),(none)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I6" xr:uid="{77C8DCE9-D337-B146-99D9-21A4944967AD}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5" xr:uid="{77C8DCE9-D337-B146-99D9-21A4944967AD}">
       <formula1>"LocalDateTime,OffsetDateTime"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2822,7 +2793,7 @@
           <x14:formula1>
             <xm:f>dropdown!$B$2:$B$20</xm:f>
           </x14:formula1>
-          <xm:sqref>N7</xm:sqref>
+          <xm:sqref>N6</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2832,7 +2803,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E1BEA4-8682-2D4B-83F3-E3D5D9773981}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.5" style="6" customWidth="1"/>
@@ -2844,7 +2815,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="B1" s="1"/>
     </row>
@@ -2854,44 +2825,33 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
+      <c r="A4" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>29</v>
-      </c>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="7"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
       <c r="D6" s="7"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="7"/>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A4:D4"/>
-  </mergeCells>
   <phoneticPr fontId="1"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C7" xr:uid="{F3EDCD97-3DDD-0A4D-ACDF-687A95CDC907}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C6" xr:uid="{F3EDCD97-3DDD-0A4D-ACDF-687A95CDC907}">
       <formula1>"quotes('),(none)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2905,7 +2865,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A480BCC2-429D-064C-9186-E29D7E93B50F}">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.5" style="6" customWidth="1"/>
@@ -2925,7 +2885,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2935,89 +2895,83 @@
       <c r="A3" s="6" t="s">
         <v>26</v>
       </c>
+      <c r="H3" s="35" t="s">
+        <v>78</v>
+      </c>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="36"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="D4" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="I4" s="33"/>
-      <c r="J4" s="33"/>
-      <c r="K4" s="33"/>
-      <c r="L4" s="33"/>
+      <c r="A4" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="H4" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="I4" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="L4" s="30" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="L5" s="8" t="s">
-        <v>39</v>
-      </c>
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8" t="str" cm="1">
+        <f t="array" ref="C5">_xlfn.IFS(テーブル3236[[#This Row],[関連テーブル処理パターン]]="論理廃止／削除","DELETE",テーブル3236[[#This Row],[関連テーブル処理パターン]]="存在チェック","CHECK_AND_SKIP_DELETE",TRUE,"")</f>
+        <v/>
+      </c>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="8"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="8"/>
-      <c r="B6" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="C6" s="8" t="str" cm="1">
-        <f t="array" ref="C6">_xlfn.IFS(テーブル3236[[#This Row],[関連テーブル処理パターン]]="論理廃止／削除","DELETE",テーブル3236[[#This Row],[関連テーブル処理パターン]]="存在チェック","CHECK_AND_SKIP_DELETE",TRUE,"")</f>
-        <v>DELETE</v>
-      </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="8"/>
+      <c r="B6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="8"/>
       <c r="B7" s="19"/>
       <c r="D7" s="19"/>
       <c r="E7" s="19"/>
-      <c r="F7" s="28"/>
+      <c r="F7" s="23"/>
       <c r="G7" s="19"/>
       <c r="H7" s="19"/>
       <c r="I7" s="19"/>
@@ -3026,51 +2980,24 @@
       <c r="L7" s="19"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="8"/>
-      <c r="B8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
+      <c r="A8" s="19"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="19" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="6" t="s">
-        <v>86</v>
-      </c>
+      <c r="A9" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="H4:L4"/>
+    <mergeCell ref="H3:L3"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G6:G8" xr:uid="{F353BD13-7B61-C54A-8C2B-F025D3AA26B4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:G7" xr:uid="{F353BD13-7B61-C54A-8C2B-F025D3AA26B4}">
       <formula1>"quotes('),(none)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:B8" xr:uid="{9B87489A-16BF-C040-BD48-9AF02F137779}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6:B7" xr:uid="{9B87489A-16BF-C040-BD48-9AF02F137779}">
       <formula1>"関連テーブル論理廃止／削除,削除対象テーブル論理廃止／削除のためのデータチェック"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6" xr:uid="{30AEF688-100C-C24A-A54E-53A83922E012}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{30AEF688-100C-C24A-A54E-53A83922E012}">
       <formula1>"論理廃止／削除,存在チェック"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>